<commit_message>
feat: atualizar arquivos binários do projeto
</commit_message>
<xml_diff>
--- a/base_cinema.xlsx
+++ b/base_cinema.xlsx
@@ -11708,17 +11708,17 @@
         <v>1</v>
       </c>
       <c r="E337" s="1"/>
-      <c r="F337" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G337" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H337" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F337" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2380.0)</f>
+        <v>2380</v>
+      </c>
+      <c r="G337" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),49.0)</f>
+        <v>49</v>
+      </c>
+      <c r="H337" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),48.57142857142857)</f>
+        <v>48.57142857</v>
       </c>
     </row>
     <row r="338">
@@ -11739,17 +11739,17 @@
         <v>2</v>
       </c>
       <c r="E338" s="1"/>
-      <c r="F338" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G338" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H338" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F338" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3015.02)</f>
+        <v>3015.02</v>
+      </c>
+      <c r="G338" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),71.0)</f>
+        <v>71</v>
+      </c>
+      <c r="H338" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.46507042253521)</f>
+        <v>42.46507042</v>
       </c>
     </row>
     <row r="339">

</xml_diff>

<commit_message>
feature: Atualização de bases
</commit_message>
<xml_diff>
--- a/base_cinema.xlsx
+++ b/base_cinema.xlsx
@@ -11770,17 +11770,17 @@
         <v>1</v>
       </c>
       <c r="E339" s="1"/>
-      <c r="F339" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G339" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H339" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F339" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3900.5)</f>
+        <v>3900.5</v>
+      </c>
+      <c r="G339" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),90.0)</f>
+        <v>90</v>
+      </c>
+      <c r="H339" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),43.33888888888889)</f>
+        <v>43.33888889</v>
       </c>
     </row>
     <row r="340">

</xml_diff>

<commit_message>
feature: atualização de dados
</commit_message>
<xml_diff>
--- a/base_cinema.xlsx
+++ b/base_cinema.xlsx
@@ -11801,17 +11801,17 @@
         <v>2</v>
       </c>
       <c r="E340" s="1"/>
-      <c r="F340" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G340" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H340" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F340" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2976.01)</f>
+        <v>2976.01</v>
+      </c>
+      <c r="G340" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),65.0)</f>
+        <v>65</v>
+      </c>
+      <c r="H340" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45.784769230769236)</f>
+        <v>45.78476923</v>
       </c>
     </row>
     <row r="341">
@@ -11832,17 +11832,17 @@
         <v>1</v>
       </c>
       <c r="E341" s="1"/>
-      <c r="F341" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G341" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H341" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F341" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),4037.5)</f>
+        <v>4037.5</v>
+      </c>
+      <c r="G341" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),89.0)</f>
+        <v>89</v>
+      </c>
+      <c r="H341" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45.36516853932584)</f>
+        <v>45.36516854</v>
       </c>
     </row>
     <row r="342">

</xml_diff>

<commit_message>
feature: Atualização de código e bases
No código foi incluído uma seção para análise de faturamento médio por dia da semana.
</commit_message>
<xml_diff>
--- a/base_cinema.xlsx
+++ b/base_cinema.xlsx
@@ -11863,17 +11863,17 @@
         <v>2</v>
       </c>
       <c r="E342" s="1"/>
-      <c r="F342" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G342" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H342" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F342" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3251.01)</f>
+        <v>3251.01</v>
+      </c>
+      <c r="G342" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),87.0)</f>
+        <v>87</v>
+      </c>
+      <c r="H342" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),37.36793103448276)</f>
+        <v>37.36793103</v>
       </c>
     </row>
     <row r="343">

</xml_diff>

<commit_message>
feature: importação de bases
</commit_message>
<xml_diff>
--- a/base_cinema.xlsx
+++ b/base_cinema.xlsx
@@ -12020,17 +12020,17 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3129.21)</f>
         <v>3129.21</v>
       </c>
-      <c r="F346" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G346" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
-      </c>
-      <c r="H346" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
+      <c r="F346" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),2524.0)</f>
+        <v>2524</v>
+      </c>
+      <c r="G346" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),47.0)</f>
+        <v>47</v>
+      </c>
+      <c r="H346" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),53.702127659574465)</f>
+        <v>53.70212766</v>
       </c>
     </row>
     <row r="347">

</xml_diff>

<commit_message>
tentativa de correções de warning
</commit_message>
<xml_diff>
--- a/base_cinema.xlsx
+++ b/base_cinema.xlsx
@@ -12462,13 +12462,13 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
         <v>0</v>
       </c>
-      <c r="F359" s="6" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>
-        <v/>
-      </c>
-      <c r="G359" s="1" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"")</f>
-        <v/>
+      <c r="F359" s="6">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
+      </c>
+      <c r="G359" s="1">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),0.0)</f>
+        <v>0</v>
       </c>
       <c r="H359" s="6" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"  ")</f>

</xml_diff>